<commit_message>
add sweeper, update metrics, fix bugs in main
</commit_message>
<xml_diff>
--- a/metrics/metrics_results.xlsx
+++ b/metrics/metrics_results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\motya\Documents\GitHub\YOLO-RAG-system\metrics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46791403-702A-4B4D-B9BC-A6CC46EA2883}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C2C4938-F7AD-482C-BE54-BD9BEC5BF3A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -149,55 +149,21 @@
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00D25F"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00D25F"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00D25F"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF00D25F"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <mruColors>
-      <color rgb="FF00D25F"/>
-    </mruColors>
-  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -497,57 +463,56 @@
   <dimension ref="A1:P6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.140625" customWidth="1"/>
-    <col min="2" max="16" width="11.7109375" customWidth="1"/>
+    <col min="1" max="16" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:16" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" s="3" t="s">
         <v>15</v>
       </c>
     </row>
@@ -555,49 +520,49 @@
       <c r="A2" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="1">
         <v>0.68</v>
       </c>
-      <c r="C2" s="3">
+      <c r="C2" s="1">
         <v>0.84</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D2" s="1">
         <v>0.84</v>
       </c>
-      <c r="E2" s="3">
+      <c r="E2" s="1">
         <v>0.32</v>
       </c>
-      <c r="F2" s="3">
+      <c r="F2" s="1">
         <v>0.52</v>
       </c>
-      <c r="G2" s="3">
+      <c r="G2" s="1">
         <v>0.52</v>
       </c>
-      <c r="H2" s="3">
+      <c r="H2" s="1">
         <v>0.6</v>
       </c>
-      <c r="I2" s="3">
+      <c r="I2" s="1">
         <v>0.76</v>
       </c>
-      <c r="J2" s="3">
+      <c r="J2" s="1">
         <v>0.76</v>
       </c>
-      <c r="K2" s="3">
+      <c r="K2" s="1">
         <v>0.64</v>
       </c>
-      <c r="L2" s="3">
+      <c r="L2" s="1">
         <v>0.72</v>
       </c>
-      <c r="M2" s="3">
+      <c r="M2" s="1">
         <v>0.72</v>
       </c>
-      <c r="N2" s="3">
+      <c r="N2" s="1">
         <v>0.64</v>
       </c>
-      <c r="O2" s="3">
+      <c r="O2" s="1">
         <v>0.76</v>
       </c>
-      <c r="P2" s="3">
+      <c r="P2" s="1">
         <v>0.76</v>
       </c>
     </row>
@@ -605,49 +570,49 @@
       <c r="A3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="1">
         <v>0.47799999999999998</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="1">
         <v>0.59</v>
       </c>
-      <c r="D3" s="3">
+      <c r="D3" s="1">
         <v>0.59</v>
       </c>
-      <c r="E3" s="3">
+      <c r="E3" s="1">
         <v>0.14299999999999999</v>
       </c>
-      <c r="F3" s="3">
+      <c r="F3" s="1">
         <v>0.35099999999999998</v>
       </c>
-      <c r="G3" s="3">
+      <c r="G3" s="1">
         <v>0.35099999999999998</v>
       </c>
-      <c r="H3" s="3">
+      <c r="H3" s="1">
         <v>0.39600000000000002</v>
       </c>
-      <c r="I3" s="3">
+      <c r="I3" s="1">
         <v>0.52100000000000002</v>
       </c>
-      <c r="J3" s="3">
+      <c r="J3" s="1">
         <v>0.52100000000000002</v>
       </c>
-      <c r="K3" s="3">
+      <c r="K3" s="1">
         <v>0.437</v>
       </c>
-      <c r="L3" s="3">
+      <c r="L3" s="1">
         <v>0.51300000000000001</v>
       </c>
-      <c r="M3" s="3">
+      <c r="M3" s="1">
         <v>0.51300000000000001</v>
       </c>
-      <c r="N3" s="3">
+      <c r="N3" s="1">
         <v>0.43099999999999999</v>
       </c>
-      <c r="O3" s="3">
+      <c r="O3" s="1">
         <v>0.55500000000000005</v>
       </c>
-      <c r="P3" s="3">
+      <c r="P3" s="1">
         <v>0.55500000000000005</v>
       </c>
     </row>
@@ -655,49 +620,49 @@
       <c r="A4" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="3">
-        <v>5</v>
-      </c>
-      <c r="C4" s="3">
-        <v>5</v>
-      </c>
-      <c r="D4" s="3">
+      <c r="B4" s="1">
+        <v>5</v>
+      </c>
+      <c r="C4" s="1">
+        <v>5</v>
+      </c>
+      <c r="D4" s="1">
         <v>4.9000000000000004</v>
       </c>
-      <c r="E4" s="3">
-        <v>5</v>
-      </c>
-      <c r="F4" s="3">
-        <v>5</v>
-      </c>
-      <c r="G4" s="3">
+      <c r="E4" s="1">
+        <v>5</v>
+      </c>
+      <c r="F4" s="1">
+        <v>5</v>
+      </c>
+      <c r="G4" s="1">
         <v>3.6</v>
       </c>
-      <c r="H4" s="3">
-        <v>5</v>
-      </c>
-      <c r="I4" s="3">
-        <v>5</v>
-      </c>
-      <c r="J4" s="3">
+      <c r="H4" s="1">
+        <v>5</v>
+      </c>
+      <c r="I4" s="1">
+        <v>5</v>
+      </c>
+      <c r="J4" s="1">
         <v>4.8</v>
       </c>
-      <c r="K4" s="3">
-        <v>5</v>
-      </c>
-      <c r="L4" s="3">
-        <v>5</v>
-      </c>
-      <c r="M4" s="3">
+      <c r="K4" s="1">
+        <v>5</v>
+      </c>
+      <c r="L4" s="1">
+        <v>5</v>
+      </c>
+      <c r="M4" s="1">
         <v>4.8</v>
       </c>
-      <c r="N4" s="3">
-        <v>5</v>
-      </c>
-      <c r="O4" s="3">
-        <v>5</v>
-      </c>
-      <c r="P4" s="3">
+      <c r="N4" s="1">
+        <v>5</v>
+      </c>
+      <c r="O4" s="1">
+        <v>5</v>
+      </c>
+      <c r="P4" s="1">
         <v>4.7</v>
       </c>
     </row>
@@ -705,129 +670,136 @@
       <c r="A5" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B5" s="3">
-        <v>4.5100000000000001E-2</v>
-      </c>
-      <c r="C5" s="3">
-        <v>0.18870000000000001</v>
-      </c>
-      <c r="D5" s="3">
-        <v>0.19869999999999999</v>
-      </c>
-      <c r="E5" s="3">
-        <v>6.7999999999999996E-3</v>
-      </c>
-      <c r="F5" s="3">
-        <v>0.16700000000000001</v>
-      </c>
-      <c r="G5" s="3">
-        <v>0.16589999999999999</v>
-      </c>
-      <c r="H5" s="3">
-        <v>6.1199999999999997E-2</v>
-      </c>
-      <c r="I5" s="3">
-        <v>0.21859999999999999</v>
-      </c>
-      <c r="J5" s="3">
-        <v>0.218</v>
-      </c>
-      <c r="K5" s="3">
-        <v>5.5800000000000002E-2</v>
-      </c>
-      <c r="L5" s="3">
-        <v>0.2177</v>
-      </c>
-      <c r="M5" s="3">
-        <v>0.21809999999999999</v>
-      </c>
-      <c r="N5" s="3">
-        <v>6.4699999999999994E-2</v>
-      </c>
-      <c r="O5" s="3">
-        <v>0.21909999999999999</v>
-      </c>
-      <c r="P5" s="3">
-        <v>0.21809999999999999</v>
+      <c r="B5" s="1">
+        <v>4.9299999999999997E-2</v>
+      </c>
+      <c r="C5" s="1">
+        <v>0.2031</v>
+      </c>
+      <c r="D5" s="1">
+        <v>0.2021</v>
+      </c>
+      <c r="E5" s="1">
+        <v>7.4000000000000003E-3</v>
+      </c>
+      <c r="F5" s="1">
+        <v>0.1744</v>
+      </c>
+      <c r="G5" s="1">
+        <v>0.17469999999999999</v>
+      </c>
+      <c r="H5" s="1">
+        <v>6.0199999999999997E-2</v>
+      </c>
+      <c r="I5" s="1">
+        <v>0.22739999999999999</v>
+      </c>
+      <c r="J5" s="1">
+        <v>0.22650000000000001</v>
+      </c>
+      <c r="K5" s="1">
+        <v>6.6900000000000001E-2</v>
+      </c>
+      <c r="L5" s="1">
+        <v>0.2281</v>
+      </c>
+      <c r="M5" s="1">
+        <v>0.2268</v>
+      </c>
+      <c r="N5" s="1">
+        <v>5.62E-2</v>
+      </c>
+      <c r="O5" s="1">
+        <v>0.23080000000000001</v>
+      </c>
+      <c r="P5" s="1">
+        <v>0.2271</v>
       </c>
     </row>
     <row r="6" spans="1:16" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B6" s="3">
-        <v>1.21E-2</v>
-      </c>
-      <c r="C6" s="3">
-        <v>3.2099999999999997E-2</v>
-      </c>
-      <c r="D6" s="3">
-        <v>2.4799999999999999E-2</v>
-      </c>
-      <c r="E6" s="3">
-        <v>2.2000000000000001E-3</v>
-      </c>
-      <c r="F6" s="3">
-        <v>3.1699999999999999E-2</v>
-      </c>
-      <c r="G6" s="3">
-        <v>3.2899999999999999E-2</v>
-      </c>
-      <c r="H6" s="3">
-        <v>1.3899999999999999E-2</v>
-      </c>
-      <c r="I6" s="3">
-        <v>3.2399999999999998E-2</v>
-      </c>
-      <c r="J6" s="3">
-        <v>3.2899999999999999E-2</v>
-      </c>
-      <c r="K6" s="3">
-        <v>1.0200000000000001E-2</v>
-      </c>
-      <c r="L6" s="3">
-        <v>3.4700000000000002E-2</v>
-      </c>
-      <c r="M6" s="3">
-        <v>3.2199999999999999E-2</v>
-      </c>
-      <c r="N6" s="3">
-        <v>1.2800000000000001E-2</v>
-      </c>
-      <c r="O6" s="3">
-        <v>3.5499999999999997E-2</v>
-      </c>
-      <c r="P6" s="3">
-        <v>3.6400000000000002E-2</v>
+      <c r="B6" s="1">
+        <v>1.0999999999999999E-2</v>
+      </c>
+      <c r="C6" s="1">
+        <v>2.06E-2</v>
+      </c>
+      <c r="D6" s="1">
+        <v>2.3699999999999999E-2</v>
+      </c>
+      <c r="E6" s="1">
+        <v>2.3E-3</v>
+      </c>
+      <c r="F6" s="1">
+        <v>3.3599999999999998E-2</v>
+      </c>
+      <c r="G6" s="1">
+        <v>3.3399999999999999E-2</v>
+      </c>
+      <c r="H6" s="1">
+        <v>1.14E-2</v>
+      </c>
+      <c r="I6" s="1">
+        <v>3.5700000000000003E-2</v>
+      </c>
+      <c r="J6" s="1">
+        <v>3.4000000000000002E-2</v>
+      </c>
+      <c r="K6" s="1">
+        <v>1.4200000000000001E-2</v>
+      </c>
+      <c r="L6" s="1">
+        <v>3.49E-2</v>
+      </c>
+      <c r="M6" s="1">
+        <v>3.2800000000000003E-2</v>
+      </c>
+      <c r="N6" s="1">
+        <v>1.01E-2</v>
+      </c>
+      <c r="O6" s="1">
+        <v>3.5400000000000001E-2</v>
+      </c>
+      <c r="P6" s="1">
+        <v>3.5000000000000003E-2</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B2:P2">
-    <cfRule type="colorScale" priority="6">
+    <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
         <cfvo type="max"/>
         <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
+        <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:P3">
-    <cfRule type="colorScale" priority="5">
+    <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
         <cfvo type="max"/>
         <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
+        <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B4:P4">
-    <cfRule type="top10" dxfId="1" priority="4" bottom="1" rank="2"/>
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFCFCFF"/>
+      </colorScale>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B5:P5">
     <cfRule type="colorScale" priority="1">
@@ -838,16 +810,6 @@
         <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="2">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
update main, metrics, add sweep parameters and update readme
</commit_message>
<xml_diff>
--- a/metrics/metrics_results.xlsx
+++ b/metrics/metrics_results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\motya\Documents\GitHub\YOLO-RAG-system\metrics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C824DF7F-338C-4456-B09D-F2526C1B7327}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C2C4938-F7AD-482C-BE54-BD9BEC5BF3A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>Метрика</t>
   </si>
@@ -85,13 +85,16 @@
   </si>
   <si>
     <t>Время (s)</t>
+  </si>
+  <si>
+    <t>Отклонение (s)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -106,12 +109,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="204"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="8"/>
-      <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -156,34 +153,17 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF7FDB91"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <mruColors>
-      <color rgb="FF7FDB91"/>
-      <color rgb="FFFFFFFF"/>
-      <color rgb="FFC6EFCE"/>
-      <color rgb="FF09FF78"/>
-      <color rgb="FF36F636"/>
-    </mruColors>
-  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -480,164 +460,164 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P5"/>
+  <dimension ref="A1:P6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="16" width="11.7109375" customWidth="1"/>
+    <col min="1" max="16" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="2" t="s">
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+      <c r="M1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="2" t="s">
+      <c r="N1" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="P1" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+    <row r="2" spans="1:16" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B2" s="1">
+        <v>0.68</v>
+      </c>
+      <c r="C2" s="1">
+        <v>0.84</v>
+      </c>
+      <c r="D2" s="1">
+        <v>0.84</v>
+      </c>
+      <c r="E2" s="1">
+        <v>0.32</v>
+      </c>
+      <c r="F2" s="1">
+        <v>0.52</v>
+      </c>
+      <c r="G2" s="1">
+        <v>0.52</v>
+      </c>
+      <c r="H2" s="1">
         <v>0.6</v>
       </c>
-      <c r="C2" s="1">
-        <v>0.8</v>
-      </c>
-      <c r="D2" s="1">
-        <v>0.8</v>
-      </c>
-      <c r="E2" s="1">
-        <v>0.28000000000000003</v>
-      </c>
-      <c r="F2" s="1">
-        <v>0.44</v>
-      </c>
-      <c r="G2" s="1">
-        <v>0.44</v>
-      </c>
-      <c r="H2" s="1">
-        <v>0.52</v>
-      </c>
       <c r="I2" s="1">
+        <v>0.76</v>
+      </c>
+      <c r="J2" s="1">
+        <v>0.76</v>
+      </c>
+      <c r="K2" s="1">
         <v>0.64</v>
       </c>
-      <c r="J2" s="1">
+      <c r="L2" s="1">
+        <v>0.72</v>
+      </c>
+      <c r="M2" s="1">
+        <v>0.72</v>
+      </c>
+      <c r="N2" s="1">
         <v>0.64</v>
       </c>
-      <c r="K2" s="1">
-        <v>0.56000000000000005</v>
-      </c>
-      <c r="L2" s="1">
-        <v>0.64</v>
-      </c>
-      <c r="M2" s="1">
-        <v>0.64</v>
-      </c>
-      <c r="N2" s="1">
-        <v>0.56000000000000005</v>
-      </c>
       <c r="O2" s="1">
-        <v>0.68</v>
+        <v>0.76</v>
       </c>
       <c r="P2" s="1">
-        <v>0.68</v>
+        <v>0.76</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+    <row r="3" spans="1:16" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
         <v>17</v>
       </c>
       <c r="B3" s="1">
-        <v>0.45100000000000001</v>
+        <v>0.47799999999999998</v>
       </c>
       <c r="C3" s="1">
-        <v>0.56999999999999995</v>
+        <v>0.59</v>
       </c>
       <c r="D3" s="1">
-        <v>0.56999999999999995</v>
+        <v>0.59</v>
       </c>
       <c r="E3" s="1">
-        <v>0.13500000000000001</v>
+        <v>0.14299999999999999</v>
       </c>
       <c r="F3" s="1">
-        <v>0.30299999999999999</v>
+        <v>0.35099999999999998</v>
       </c>
       <c r="G3" s="1">
-        <v>0.30299999999999999</v>
+        <v>0.35099999999999998</v>
       </c>
       <c r="H3" s="1">
-        <v>0.36799999999999999</v>
+        <v>0.39600000000000002</v>
       </c>
       <c r="I3" s="1">
-        <v>0.47299999999999998</v>
+        <v>0.52100000000000002</v>
       </c>
       <c r="J3" s="1">
-        <v>0.47299999999999998</v>
+        <v>0.52100000000000002</v>
       </c>
       <c r="K3" s="1">
-        <v>0.41599999999999998</v>
+        <v>0.437</v>
       </c>
       <c r="L3" s="1">
-        <v>0.47299999999999998</v>
+        <v>0.51300000000000001</v>
       </c>
       <c r="M3" s="1">
-        <v>0.47299999999999998</v>
+        <v>0.51300000000000001</v>
       </c>
       <c r="N3" s="1">
-        <v>0.40100000000000002</v>
+        <v>0.43099999999999999</v>
       </c>
       <c r="O3" s="1">
-        <v>0.51500000000000001</v>
+        <v>0.55500000000000005</v>
       </c>
       <c r="P3" s="1">
-        <v>0.51500000000000001</v>
+        <v>0.55500000000000005</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+    <row r="4" spans="1:16" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
         <v>18</v>
       </c>
       <c r="B4" s="1">
@@ -647,129 +627,187 @@
         <v>5</v>
       </c>
       <c r="D4" s="1">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="E4" s="1">
+        <v>5</v>
+      </c>
+      <c r="F4" s="1">
+        <v>5</v>
+      </c>
+      <c r="G4" s="1">
+        <v>3.6</v>
+      </c>
+      <c r="H4" s="1">
+        <v>5</v>
+      </c>
+      <c r="I4" s="1">
+        <v>5</v>
+      </c>
+      <c r="J4" s="1">
         <v>4.8</v>
       </c>
-      <c r="E4" s="1">
-        <v>5</v>
-      </c>
-      <c r="F4" s="1">
-        <v>5</v>
-      </c>
-      <c r="G4" s="1">
-        <v>3.2</v>
-      </c>
-      <c r="H4" s="1">
-        <v>5</v>
-      </c>
-      <c r="I4" s="1">
-        <v>5</v>
-      </c>
-      <c r="J4" s="1">
+      <c r="K4" s="1">
+        <v>5</v>
+      </c>
+      <c r="L4" s="1">
+        <v>5</v>
+      </c>
+      <c r="M4" s="1">
+        <v>4.8</v>
+      </c>
+      <c r="N4" s="1">
+        <v>5</v>
+      </c>
+      <c r="O4" s="1">
+        <v>5</v>
+      </c>
+      <c r="P4" s="1">
         <v>4.7</v>
       </c>
-      <c r="K4" s="1">
-        <v>5</v>
-      </c>
-      <c r="L4" s="1">
-        <v>5</v>
-      </c>
-      <c r="M4" s="1">
-        <v>4.7</v>
-      </c>
-      <c r="N4" s="1">
-        <v>5</v>
-      </c>
-      <c r="O4" s="1">
-        <v>5</v>
-      </c>
-      <c r="P4" s="1">
-        <v>4.5999999999999996</v>
-      </c>
     </row>
-    <row r="5" spans="1:16" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+    <row r="5" spans="1:16" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
         <v>19</v>
       </c>
       <c r="B5" s="1">
-        <v>5.6099999999999997E-2</v>
+        <v>4.9299999999999997E-2</v>
       </c>
       <c r="C5" s="1">
-        <v>0.1956</v>
+        <v>0.2031</v>
       </c>
       <c r="D5" s="1">
-        <v>0.1958</v>
+        <v>0.2021</v>
       </c>
       <c r="E5" s="1">
-        <v>8.5000000000000006E-3</v>
+        <v>7.4000000000000003E-3</v>
       </c>
       <c r="F5" s="1">
-        <v>0.17199999999999999</v>
+        <v>0.1744</v>
       </c>
       <c r="G5" s="1">
-        <v>0.1792</v>
+        <v>0.17469999999999999</v>
       </c>
       <c r="H5" s="1">
-        <v>6.2300000000000001E-2</v>
+        <v>6.0199999999999997E-2</v>
       </c>
       <c r="I5" s="1">
-        <v>0.23780000000000001</v>
+        <v>0.22739999999999999</v>
       </c>
       <c r="J5" s="1">
-        <v>0.23599999999999999</v>
+        <v>0.22650000000000001</v>
       </c>
       <c r="K5" s="1">
-        <v>7.22E-2</v>
+        <v>6.6900000000000001E-2</v>
       </c>
       <c r="L5" s="1">
-        <v>0.23419999999999999</v>
+        <v>0.2281</v>
       </c>
       <c r="M5" s="1">
-        <v>0.22259999999999999</v>
+        <v>0.2268</v>
       </c>
       <c r="N5" s="1">
-        <v>6.3500000000000001E-2</v>
+        <v>5.62E-2</v>
       </c>
       <c r="O5" s="1">
-        <v>0.21859999999999999</v>
+        <v>0.23080000000000001</v>
       </c>
       <c r="P5" s="1">
-        <v>0.23469999999999999</v>
+        <v>0.2271</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="1">
+        <v>1.0999999999999999E-2</v>
+      </c>
+      <c r="C6" s="1">
+        <v>2.06E-2</v>
+      </c>
+      <c r="D6" s="1">
+        <v>2.3699999999999999E-2</v>
+      </c>
+      <c r="E6" s="1">
+        <v>2.3E-3</v>
+      </c>
+      <c r="F6" s="1">
+        <v>3.3599999999999998E-2</v>
+      </c>
+      <c r="G6" s="1">
+        <v>3.3399999999999999E-2</v>
+      </c>
+      <c r="H6" s="1">
+        <v>1.14E-2</v>
+      </c>
+      <c r="I6" s="1">
+        <v>3.5700000000000003E-2</v>
+      </c>
+      <c r="J6" s="1">
+        <v>3.4000000000000002E-2</v>
+      </c>
+      <c r="K6" s="1">
+        <v>1.4200000000000001E-2</v>
+      </c>
+      <c r="L6" s="1">
+        <v>3.49E-2</v>
+      </c>
+      <c r="M6" s="1">
+        <v>3.2800000000000003E-2</v>
+      </c>
+      <c r="N6" s="1">
+        <v>1.01E-2</v>
+      </c>
+      <c r="O6" s="1">
+        <v>3.5400000000000001E-2</v>
+      </c>
+      <c r="P6" s="1">
+        <v>3.5000000000000003E-2</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="2" type="noConversion"/>
   <conditionalFormatting sqref="B2:P2">
-    <cfRule type="colorScale" priority="2">
+    <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
         <cfvo type="max"/>
-        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:P3">
-    <cfRule type="colorScale" priority="1">
+    <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
         <cfvo type="max"/>
-        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
         <color rgb="FF63BE7B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B4:P4">
-    <cfRule type="top10" dxfId="0" priority="6" bottom="1" rank="2"/>
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFCFCFF"/>
+      </colorScale>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B5:P5">
-    <cfRule type="colorScale" priority="3">
+    <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
         <cfvo type="max"/>
         <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>

</xml_diff>